<commit_message>
feat: Add CSV bulk upload functionality for master data
Add CSV upload components for ingredients, menus, and SKUs to enable efficient bulk data import.

🤖 Generated with [Claude Code](https://claude.com/claude-code)

Co-Authored-By: Claude Sonnet 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/매입_판매_원가.xlsx
+++ b/매입_판매_원가.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\내 드라이브\오프라인용\나성닭강정\매출\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\내 드라이브\오프라인용\나성닭강정\매입_판매_원가\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A7D969F5-BF60-4D35-A70D-5FA143F22906}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26DD29AB-D1BF-4281-A759-474DE13301B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29940" yWindow="1140" windowWidth="21600" windowHeight="11175" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="사용안내" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,6 @@
     <definedName name="붕어빵">범례!$C$2:$C$11</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -48,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1611" uniqueCount="144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1615" uniqueCount="145">
   <si>
     <t>매입·판매수량 기록 템플릿 사용 안내</t>
   </si>
@@ -480,6 +479,10 @@
   </si>
   <si>
     <t>* '기준단위당 원가'는 [환산계수]로 환산한 기준단위(예: 닭강정=컵환산) 기준 평균원가입니다.</t>
+  </si>
+  <si>
+    <t>황금잉어빵본사</t>
+    <phoneticPr fontId="7" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -913,6 +916,12 @@
     <xf numFmtId="0" fontId="11" fillId="13" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="5" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -927,12 +936,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1157,79 +1160,79 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="53" t="s">
+      <c r="A1" s="55" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="54"/>
-      <c r="C1" s="54"/>
-      <c r="D1" s="54"/>
-      <c r="E1" s="54"/>
-      <c r="F1" s="54"/>
-      <c r="G1" s="54"/>
-      <c r="H1" s="54"/>
+      <c r="B1" s="56"/>
+      <c r="C1" s="56"/>
+      <c r="D1" s="56"/>
+      <c r="E1" s="56"/>
+      <c r="F1" s="56"/>
+      <c r="G1" s="56"/>
+      <c r="H1" s="56"/>
     </row>
     <row r="3" spans="1:8" ht="39.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="60" t="s">
+      <c r="A3" s="53" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="61"/>
-      <c r="C3" s="61"/>
-      <c r="D3" s="61"/>
-      <c r="E3" s="61"/>
-      <c r="F3" s="61"/>
-      <c r="G3" s="61"/>
-      <c r="H3" s="61"/>
+      <c r="B3" s="54"/>
+      <c r="C3" s="54"/>
+      <c r="D3" s="54"/>
+      <c r="E3" s="54"/>
+      <c r="F3" s="54"/>
+      <c r="G3" s="54"/>
+      <c r="H3" s="54"/>
     </row>
     <row r="4" spans="1:8" ht="39.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="60" t="s">
+      <c r="A4" s="53" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="61"/>
-      <c r="C4" s="61"/>
-      <c r="D4" s="61"/>
-      <c r="E4" s="61"/>
-      <c r="F4" s="61"/>
-      <c r="G4" s="61"/>
-      <c r="H4" s="61"/>
+      <c r="B4" s="54"/>
+      <c r="C4" s="54"/>
+      <c r="D4" s="54"/>
+      <c r="E4" s="54"/>
+      <c r="F4" s="54"/>
+      <c r="G4" s="54"/>
+      <c r="H4" s="54"/>
     </row>
     <row r="5" spans="1:8" ht="39.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="60" t="s">
+      <c r="A5" s="53" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="61"/>
-      <c r="C5" s="61"/>
-      <c r="D5" s="61"/>
-      <c r="E5" s="61"/>
-      <c r="F5" s="61"/>
-      <c r="G5" s="61"/>
-      <c r="H5" s="61"/>
+      <c r="B5" s="54"/>
+      <c r="C5" s="54"/>
+      <c r="D5" s="54"/>
+      <c r="E5" s="54"/>
+      <c r="F5" s="54"/>
+      <c r="G5" s="54"/>
+      <c r="H5" s="54"/>
     </row>
     <row r="6" spans="1:8" ht="39.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="60" t="s">
+      <c r="A6" s="53" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="61"/>
-      <c r="C6" s="61"/>
-      <c r="D6" s="61"/>
-      <c r="E6" s="61"/>
-      <c r="F6" s="61"/>
-      <c r="G6" s="61"/>
-      <c r="H6" s="61"/>
+      <c r="B6" s="54"/>
+      <c r="C6" s="54"/>
+      <c r="D6" s="54"/>
+      <c r="E6" s="54"/>
+      <c r="F6" s="54"/>
+      <c r="G6" s="54"/>
+      <c r="H6" s="54"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" s="1"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A8" s="60" t="s">
+      <c r="A8" s="53" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="61"/>
-      <c r="C8" s="61"/>
-      <c r="D8" s="61"/>
-      <c r="E8" s="61"/>
-      <c r="F8" s="61"/>
-      <c r="G8" s="61"/>
-      <c r="H8" s="61"/>
+      <c r="B8" s="54"/>
+      <c r="C8" s="54"/>
+      <c r="D8" s="54"/>
+      <c r="E8" s="54"/>
+      <c r="F8" s="54"/>
+      <c r="G8" s="54"/>
+      <c r="H8" s="54"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" s="1"/>
@@ -8961,87 +8964,119 @@
       </c>
     </row>
     <row r="231" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A231" s="39"/>
+      <c r="A231" s="39">
+        <v>46027</v>
+      </c>
       <c r="B231" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="C231" s="40"/>
+      <c r="C231" s="40" t="s">
+        <v>62</v>
+      </c>
       <c r="D231" s="41" t="s">
-        <v>77</v>
-      </c>
-      <c r="E231" s="40"/>
-      <c r="F231" s="40"/>
-      <c r="G231" s="42" t="str">
+        <v>144</v>
+      </c>
+      <c r="E231" s="40">
+        <v>1</v>
+      </c>
+      <c r="F231" s="40">
+        <v>8500</v>
+      </c>
+      <c r="G231" s="42">
         <f t="shared" si="3"/>
-        <v/>
+        <v>8500</v>
       </c>
       <c r="H231" s="40"/>
       <c r="I231" s="43" t="str">
         <f>IF(OR(B231="",C231=""),"",IF(COUNTIFS(재료목록!$A$2:$A$51,B231,재료목록!$B$2:$B$51,C231)&gt;0,"OK","불일치"))</f>
-        <v/>
+        <v>OK</v>
       </c>
     </row>
     <row r="232" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A232" s="39"/>
+      <c r="A232" s="39">
+        <v>46027</v>
+      </c>
       <c r="B232" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="C232" s="40"/>
+      <c r="C232" s="40" t="s">
+        <v>48</v>
+      </c>
       <c r="D232" s="41" t="s">
         <v>77</v>
       </c>
-      <c r="E232" s="40"/>
-      <c r="F232" s="40"/>
-      <c r="G232" s="42" t="str">
+      <c r="E232" s="40">
+        <v>2</v>
+      </c>
+      <c r="F232" s="40">
+        <v>13000</v>
+      </c>
+      <c r="G232" s="42">
         <f t="shared" si="3"/>
-        <v/>
+        <v>26000</v>
       </c>
       <c r="H232" s="40"/>
       <c r="I232" s="43" t="str">
         <f>IF(OR(B232="",C232=""),"",IF(COUNTIFS(재료목록!$A$2:$A$51,B232,재료목록!$B$2:$B$51,C232)&gt;0,"OK","불일치"))</f>
-        <v/>
+        <v>OK</v>
       </c>
     </row>
     <row r="233" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A233" s="39"/>
+      <c r="A233" s="39">
+        <v>46027</v>
+      </c>
       <c r="B233" s="40" t="s">
-        <v>22</v>
-      </c>
-      <c r="C233" s="40"/>
+        <v>11</v>
+      </c>
+      <c r="C233" s="40" t="s">
+        <v>26</v>
+      </c>
       <c r="D233" s="41" t="s">
         <v>77</v>
       </c>
-      <c r="E233" s="40"/>
-      <c r="F233" s="40"/>
-      <c r="G233" s="42" t="str">
+      <c r="E233" s="40">
+        <v>1</v>
+      </c>
+      <c r="F233" s="40">
+        <v>8000</v>
+      </c>
+      <c r="G233" s="42">
         <f t="shared" si="3"/>
-        <v/>
+        <v>8000</v>
       </c>
       <c r="H233" s="40"/>
       <c r="I233" s="43" t="str">
         <f>IF(OR(B233="",C233=""),"",IF(COUNTIFS(재료목록!$A$2:$A$51,B233,재료목록!$B$2:$B$51,C233)&gt;0,"OK","불일치"))</f>
-        <v/>
+        <v>OK</v>
       </c>
     </row>
     <row r="234" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A234" s="39"/>
+      <c r="A234" s="39">
+        <v>46027</v>
+      </c>
       <c r="B234" s="40" t="s">
-        <v>22</v>
-      </c>
-      <c r="C234" s="40"/>
+        <v>16</v>
+      </c>
+      <c r="C234" s="40" t="s">
+        <v>47</v>
+      </c>
       <c r="D234" s="41" t="s">
         <v>77</v>
       </c>
-      <c r="E234" s="40"/>
-      <c r="F234" s="40"/>
-      <c r="G234" s="42" t="str">
+      <c r="E234" s="40">
+        <v>1</v>
+      </c>
+      <c r="F234" s="40">
+        <v>8000</v>
+      </c>
+      <c r="G234" s="42">
         <f t="shared" si="3"/>
-        <v/>
+        <v>8000</v>
       </c>
       <c r="H234" s="40"/>
       <c r="I234" s="43" t="str">
         <f>IF(OR(B234="",C234=""),"",IF(COUNTIFS(재료목록!$A$2:$A$51,B234,재료목록!$B$2:$B$51,C234)&gt;0,"OK","불일치"))</f>
-        <v/>
+        <v>OK</v>
       </c>
     </row>
     <row r="235" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.35">
@@ -14815,7 +14850,7 @@
       <c r="E514" s="40"/>
       <c r="F514" s="40"/>
       <c r="G514" s="42" t="str">
-        <f t="shared" ref="G514:G577" si="8">IF(OR(E514="",F514=""),"",E514*F514)</f>
+        <f t="shared" ref="G514:G561" si="8">IF(OR(E514="",F514=""),"",E514*F514)</f>
         <v/>
       </c>
       <c r="H514" s="40"/>
@@ -15736,6 +15771,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -22066,16 +22102,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="55" t="s">
+      <c r="A1" s="57" t="s">
         <v>123</v>
       </c>
-      <c r="B1" s="54"/>
-      <c r="C1" s="54"/>
-      <c r="D1" s="54"/>
-      <c r="E1" s="54"/>
-      <c r="F1" s="54"/>
-      <c r="G1" s="54"/>
-      <c r="H1" s="54"/>
+      <c r="B1" s="56"/>
+      <c r="C1" s="56"/>
+      <c r="D1" s="56"/>
+      <c r="E1" s="56"/>
+      <c r="F1" s="56"/>
+      <c r="G1" s="56"/>
+      <c r="H1" s="56"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" s="7" t="s">
@@ -22094,17 +22130,17 @@
       </c>
     </row>
     <row r="6" spans="1:9" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="56" t="s">
+      <c r="A6" s="58" t="s">
         <v>126</v>
       </c>
-      <c r="B6" s="57"/>
-      <c r="C6" s="57"/>
-      <c r="D6" s="58"/>
-      <c r="F6" s="56" t="s">
+      <c r="B6" s="59"/>
+      <c r="C6" s="59"/>
+      <c r="D6" s="60"/>
+      <c r="F6" s="58" t="s">
         <v>127</v>
       </c>
-      <c r="G6" s="57"/>
-      <c r="H6" s="58"/>
+      <c r="G6" s="59"/>
+      <c r="H6" s="60"/>
     </row>
     <row r="7" spans="1:9" ht="14.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
@@ -22261,13 +22297,13 @@
       </c>
     </row>
     <row r="14" spans="1:9" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="56" t="s">
+      <c r="A14" s="58" t="s">
         <v>133</v>
       </c>
-      <c r="B14" s="57"/>
-      <c r="C14" s="57"/>
-      <c r="D14" s="57"/>
-      <c r="E14" s="58"/>
+      <c r="B14" s="59"/>
+      <c r="C14" s="59"/>
+      <c r="D14" s="59"/>
+      <c r="E14" s="60"/>
     </row>
     <row r="15" spans="1:9" ht="14.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
@@ -22467,14 +22503,14 @@
       </c>
     </row>
     <row r="27" spans="1:6" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="56" t="s">
+      <c r="A27" s="58" t="s">
         <v>137</v>
       </c>
-      <c r="B27" s="57"/>
-      <c r="C27" s="57"/>
-      <c r="D27" s="57"/>
-      <c r="E27" s="57"/>
-      <c r="F27" s="58"/>
+      <c r="B27" s="59"/>
+      <c r="C27" s="59"/>
+      <c r="D27" s="59"/>
+      <c r="E27" s="59"/>
+      <c r="F27" s="60"/>
     </row>
     <row r="28" spans="1:6" ht="14.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
@@ -22593,14 +22629,14 @@
       </c>
     </row>
     <row r="34" spans="1:6" ht="22.65" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="59" t="s">
+      <c r="A34" s="61" t="s">
         <v>143</v>
       </c>
-      <c r="B34" s="54"/>
-      <c r="C34" s="54"/>
-      <c r="D34" s="54"/>
-      <c r="E34" s="54"/>
-      <c r="F34" s="54"/>
+      <c r="B34" s="56"/>
+      <c r="C34" s="56"/>
+      <c r="D34" s="56"/>
+      <c r="E34" s="56"/>
+      <c r="F34" s="56"/>
     </row>
   </sheetData>
   <mergeCells count="6">

</xml_diff>

<commit_message>
debug: Add detailed cost calculation debugging tools
- Add debug-actions.ts with step-by-step data inspection
- Add /dashboard/analysis/debug page to view debug output
- Add console logs to main getAnalysis function
- This helps diagnose why costs are showing as 0
</commit_message>
<xml_diff>
--- a/매입_판매_원가.xlsx
+++ b/매입_판매_원가.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\내 드라이브\오프라인용\나성닭강정\매입_판매_원가\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26DD29AB-D1BF-4281-A759-474DE13301B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{674ADC5E-6B28-48A7-993B-557CAAD0C41F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="사용안내" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1615" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1615" uniqueCount="153">
   <si>
     <t>매입·판매수량 기록 템플릿 사용 안내</t>
   </si>
@@ -484,6 +484,224 @@
     <t>황금잉어빵본사</t>
     <phoneticPr fontId="7" type="noConversion"/>
   </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>닭강정</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>_</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+      </rPr>
+      <t>소</t>
+    </r>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>닭강정</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>_</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>중</t>
+    </r>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>떡볶이</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>_</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>컵</t>
+    </r>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>떡볶이</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>_</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>1인분</t>
+    </r>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>꼬치오뎅</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>붕어빵</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>3</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+      </rPr>
+      <t>마리</t>
+    </r>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>붕어빵</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>1</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+      </rPr>
+      <t>마리</t>
+    </r>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>모짜렐라붕어빵</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
@@ -493,7 +711,7 @@
     <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd"/>
     <numFmt numFmtId="177" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="20" x14ac:knownFonts="1">
+  <fonts count="23" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -625,6 +843,30 @@
       <sz val="13"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="맑은 고딕"/>
+      <family val="2"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="3"/>
+      <charset val="129"/>
     </font>
   </fonts>
   <fills count="14">
@@ -780,7 +1022,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -936,6 +1178,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="5" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="5" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -15783,7 +16031,8 @@
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="13" customWidth="1"/>
     <col min="3" max="3" width="13" bestFit="1" customWidth="1"/>
-    <col min="4" max="10" width="13" customWidth="1"/>
+    <col min="4" max="9" width="13" customWidth="1"/>
+    <col min="10" max="10" width="16.26953125" customWidth="1"/>
     <col min="11" max="11" width="15" customWidth="1"/>
   </cols>
   <sheetData>
@@ -15794,29 +16043,29 @@
       <c r="B1" s="17" t="s">
         <v>99</v>
       </c>
-      <c r="C1" s="17" t="s">
-        <v>100</v>
-      </c>
-      <c r="D1" s="17" t="s">
-        <v>101</v>
-      </c>
-      <c r="E1" s="17" t="s">
-        <v>102</v>
-      </c>
-      <c r="F1" s="17" t="s">
-        <v>103</v>
-      </c>
-      <c r="G1" s="17" t="s">
-        <v>104</v>
-      </c>
-      <c r="H1" s="17" t="s">
-        <v>105</v>
-      </c>
-      <c r="I1" s="17" t="s">
-        <v>106</v>
-      </c>
-      <c r="J1" s="17" t="s">
-        <v>107</v>
+      <c r="C1" s="62" t="s">
+        <v>145</v>
+      </c>
+      <c r="D1" s="62" t="s">
+        <v>146</v>
+      </c>
+      <c r="E1" s="62" t="s">
+        <v>147</v>
+      </c>
+      <c r="F1" s="62" t="s">
+        <v>148</v>
+      </c>
+      <c r="G1" s="63" t="s">
+        <v>149</v>
+      </c>
+      <c r="H1" s="62" t="s">
+        <v>150</v>
+      </c>
+      <c r="I1" s="62" t="s">
+        <v>151</v>
+      </c>
+      <c r="J1" s="63" t="s">
+        <v>152</v>
       </c>
       <c r="K1" s="17" t="s">
         <v>71</v>
@@ -17734,15 +17983,33 @@
       <c r="A86" s="39">
         <v>46027</v>
       </c>
-      <c r="B86" s="46"/>
-      <c r="C86" s="46"/>
-      <c r="D86" s="46"/>
-      <c r="E86" s="46"/>
-      <c r="F86" s="46"/>
-      <c r="G86" s="46"/>
-      <c r="H86" s="46"/>
-      <c r="I86" s="46"/>
-      <c r="J86" s="46"/>
+      <c r="B86" s="46">
+        <v>17</v>
+      </c>
+      <c r="C86" s="46">
+        <v>3</v>
+      </c>
+      <c r="D86" s="46">
+        <v>1</v>
+      </c>
+      <c r="E86" s="46">
+        <v>9</v>
+      </c>
+      <c r="F86" s="46">
+        <v>3</v>
+      </c>
+      <c r="G86" s="46">
+        <v>42</v>
+      </c>
+      <c r="H86" s="46">
+        <v>52</v>
+      </c>
+      <c r="I86" s="46">
+        <v>8</v>
+      </c>
+      <c r="J86" s="46">
+        <v>15</v>
+      </c>
       <c r="K86" s="47"/>
     </row>
     <row r="87" spans="1:11" x14ac:dyDescent="0.35">
@@ -22118,7 +22385,7 @@
         <v>124</v>
       </c>
       <c r="B3" s="8">
-        <v>45992</v>
+        <v>45931</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.35">
@@ -22126,7 +22393,7 @@
         <v>125</v>
       </c>
       <c r="B4" s="8">
-        <v>46022</v>
+        <v>46027</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -22174,7 +22441,7 @@
       </c>
       <c r="B8" s="9">
         <f>IF(SUM(매입현황_기록!$G$5:$G$561)=0,"",SUMIFS(매입현황_기록!$G$5:$G$561,매입현황_기록!$B$5:$B$561,"닭강정",매입현황_기록!$A$5:$A$561,"&gt;="&amp;$B$3,매입현황_기록!$A$5:$A$561,"&lt;="&amp;$B$4))</f>
-        <v>774000</v>
+        <v>1517660</v>
       </c>
       <c r="C8" s="9">
         <f>H8</f>
@@ -22182,7 +22449,7 @@
       </c>
       <c r="D8" s="9">
         <f>B8+C8</f>
-        <v>774000</v>
+        <v>1517660</v>
       </c>
       <c r="F8" s="4" t="s">
         <v>11</v>
@@ -22205,7 +22472,7 @@
       </c>
       <c r="B9" s="9">
         <f>IF(SUM(매입현황_기록!$G$5:$G$561)=0,"",SUMIFS(매입현황_기록!$G$5:$G$561,매입현황_기록!$B$5:$B$561,"떡볶이",매입현황_기록!$A$5:$A$561,"&gt;="&amp;$B$3,매입현황_기록!$A$5:$A$561,"&lt;="&amp;$B$4))</f>
-        <v>271000</v>
+        <v>499000</v>
       </c>
       <c r="C9" s="9">
         <f>H9</f>
@@ -22213,7 +22480,7 @@
       </c>
       <c r="D9" s="9">
         <f>B9+C9</f>
-        <v>271000</v>
+        <v>499000</v>
       </c>
       <c r="F9" s="4" t="s">
         <v>16</v>
@@ -22232,7 +22499,7 @@
       </c>
       <c r="B10" s="9">
         <f>IF(SUM(매입현황_기록!$G$5:$G$561)=0,"",SUMIFS(매입현황_기록!$G$5:$G$561,매입현황_기록!$B$5:$B$561,"꼬치오뎅",매입현황_기록!$A$5:$A$561,"&gt;="&amp;$B$3,매입현황_기록!$A$5:$A$561,"&lt;="&amp;$B$4))</f>
-        <v>194000</v>
+        <v>482400</v>
       </c>
       <c r="C10" s="9">
         <f>H10</f>
@@ -22240,7 +22507,7 @@
       </c>
       <c r="D10" s="9">
         <f>B10+C10</f>
-        <v>194000</v>
+        <v>482400</v>
       </c>
       <c r="F10" s="4" t="s">
         <v>19</v>
@@ -22259,7 +22526,7 @@
       </c>
       <c r="B11" s="9">
         <f>IF(SUM(매입현황_기록!$G$5:$G$561)=0,"",SUMIFS(매입현황_기록!$G$5:$G$561,매입현황_기록!$B$5:$B$561,"붕어빵",매입현황_기록!$A$5:$A$561,"&gt;="&amp;$B$3,매입현황_기록!$A$5:$A$561,"&lt;="&amp;$B$4))</f>
-        <v>904490</v>
+        <v>2658590</v>
       </c>
       <c r="C11" s="9">
         <f>H11</f>
@@ -22267,7 +22534,7 @@
       </c>
       <c r="D11" s="9">
         <f>B11+C11</f>
-        <v>904490</v>
+        <v>2658590</v>
       </c>
       <c r="F11" s="4" t="s">
         <v>22</v>
@@ -22331,7 +22598,7 @@
       </c>
       <c r="C16" s="6">
         <f>IF(SUM(판매수량_기록!$B$2:$B$399)=0,"",SUMIFS(판매수량_기록!$B$2:$B$399,판매수량_기록!$A$2:$A$399,"&gt;="&amp;$B$3,판매수량_기록!$A$2:$A$399,"&lt;="&amp;$B$4))</f>
-        <v>414</v>
+        <v>445</v>
       </c>
       <c r="D16" s="12">
         <f>환산계수!$D$2</f>
@@ -22339,7 +22606,7 @@
       </c>
       <c r="E16" s="12">
         <f t="shared" ref="E16:E24" si="0">C16*D16</f>
-        <v>414</v>
+        <v>445</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.35">
@@ -22351,7 +22618,7 @@
       </c>
       <c r="C17" s="6">
         <f>IF(SUM(판매수량_기록!$C$2:$C$399)=0,"",SUMIFS(판매수량_기록!$C$2:$C$399,판매수량_기록!$A$2:$A$399,"&gt;="&amp;$B$3,판매수량_기록!$A$2:$A$399,"&lt;="&amp;$B$4))</f>
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="D17" s="12">
         <f>환산계수!$D$3</f>
@@ -22359,7 +22626,7 @@
       </c>
       <c r="E17" s="12">
         <f t="shared" si="0"/>
-        <v>227.2</v>
+        <v>258.44</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.35">
@@ -22371,7 +22638,7 @@
       </c>
       <c r="C18" s="6">
         <f>IF(SUM(판매수량_기록!$D$2:$D$399)=0,"",SUMIFS(판매수량_기록!$D$2:$D$399,판매수량_기록!$A$2:$A$399,"&gt;="&amp;$B$3,판매수량_기록!$A$2:$A$399,"&lt;="&amp;$B$4))</f>
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="D18" s="12">
         <f>환산계수!$D$4</f>
@@ -22379,7 +22646,7 @@
       </c>
       <c r="E18" s="12">
         <f t="shared" si="0"/>
-        <v>77.44</v>
+        <v>101.64</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.35">
@@ -22391,7 +22658,7 @@
       </c>
       <c r="C19" s="6">
         <f>IF(SUM(판매수량_기록!$E$2:$E$399)=0,"",SUMIFS(판매수량_기록!$E$2:$E$399,판매수량_기록!$A$2:$A$399,"&gt;="&amp;$B$3,판매수량_기록!$A$2:$A$399,"&lt;="&amp;$B$4))</f>
-        <v>184</v>
+        <v>203</v>
       </c>
       <c r="D19" s="12">
         <f>환산계수!$D$5</f>
@@ -22399,7 +22666,7 @@
       </c>
       <c r="E19" s="12">
         <f t="shared" si="0"/>
-        <v>184</v>
+        <v>203</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.35">
@@ -22411,7 +22678,7 @@
       </c>
       <c r="C20" s="6">
         <f>IF(SUM(판매수량_기록!$F$2:$F$399)=0,"",SUMIFS(판매수량_기록!$F$2:$F$399,판매수량_기록!$A$2:$A$399,"&gt;="&amp;$B$3,판매수량_기록!$A$2:$A$399,"&lt;="&amp;$B$4))</f>
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="D20" s="12">
         <f>환산계수!$D$6</f>
@@ -22419,7 +22686,7 @@
       </c>
       <c r="E20" s="12">
         <f t="shared" si="0"/>
-        <v>210</v>
+        <v>228</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.35">
@@ -22431,7 +22698,7 @@
       </c>
       <c r="C21" s="6">
         <f>IF(SUM(판매수량_기록!$G$2:$G$399)=0,"",SUMIFS(판매수량_기록!$G$2:$G$399,판매수량_기록!$A$2:$A$399,"&gt;="&amp;$B$3,판매수량_기록!$A$2:$A$399,"&lt;="&amp;$B$4))</f>
-        <v>652</v>
+        <v>738</v>
       </c>
       <c r="D21" s="12">
         <f>환산계수!$D$7</f>
@@ -22439,7 +22706,7 @@
       </c>
       <c r="E21" s="12">
         <f t="shared" si="0"/>
-        <v>652</v>
+        <v>738</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.35">
@@ -22451,7 +22718,7 @@
       </c>
       <c r="C22" s="6">
         <f>IF(SUM(판매수량_기록!$H$2:$H$399)=0,"",SUMIFS(판매수량_기록!$H$2:$H$399,판매수량_기록!$A$2:$A$399,"&gt;="&amp;$B$3,판매수량_기록!$A$2:$A$399,"&lt;="&amp;$B$4))</f>
-        <v>1673</v>
+        <v>5727</v>
       </c>
       <c r="D22" s="12">
         <f>환산계수!$D$8</f>
@@ -22459,7 +22726,7 @@
       </c>
       <c r="E22" s="12">
         <f t="shared" si="0"/>
-        <v>1673</v>
+        <v>5727</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.35">
@@ -22471,7 +22738,7 @@
       </c>
       <c r="C23" s="6">
         <f>IF(SUM(판매수량_기록!$I$2:$I$399)=0,"",SUMIFS(판매수량_기록!$I$2:$I$399,판매수량_기록!$A$2:$A$399,"&gt;="&amp;$B$3,판매수량_기록!$A$2:$A$399,"&lt;="&amp;$B$4))</f>
-        <v>1998</v>
+        <v>6625</v>
       </c>
       <c r="D23" s="12">
         <f>환산계수!$D$9</f>
@@ -22479,7 +22746,7 @@
       </c>
       <c r="E23" s="12">
         <f t="shared" si="0"/>
-        <v>1998</v>
+        <v>6625</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.35">
@@ -22491,7 +22758,7 @@
       </c>
       <c r="C24" s="6">
         <f>IF(SUM(판매수량_기록!$J$2:$J$399)=0,"",SUMIFS(판매수량_기록!$J$2:$J$399,판매수량_기록!$A$2:$A$399,"&gt;="&amp;$B$3,판매수량_기록!$A$2:$A$399,"&lt;="&amp;$B$4))</f>
-        <v>42</v>
+        <v>79</v>
       </c>
       <c r="D24" s="12">
         <f>환산계수!$D$10</f>
@@ -22499,7 +22766,7 @@
       </c>
       <c r="E24" s="12">
         <f t="shared" si="0"/>
-        <v>63</v>
+        <v>118.5</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -22538,22 +22805,22 @@
       </c>
       <c r="B29" s="14">
         <f>SUMIFS($E$16:$E$24,$B$16:$B$24,"닭강정")</f>
-        <v>718.6400000000001</v>
+        <v>805.08</v>
       </c>
       <c r="C29" s="9">
         <f>$D$8</f>
-        <v>774000</v>
+        <v>1517660</v>
       </c>
       <c r="D29" s="9">
         <f>IF(B29=0,"",C29/B29)</f>
-        <v>1077.0343983079149</v>
+        <v>1885.104585879664</v>
       </c>
       <c r="E29" s="15">
-        <v>2241563</v>
+        <v>7565461</v>
       </c>
       <c r="F29" s="16">
         <f>IFERROR( (E29 - (B29*D29)) / E29, "" )</f>
-        <v>0.65470522131209341</v>
+        <v>0.79939622978692249</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.35">
@@ -22562,22 +22829,22 @@
       </c>
       <c r="B30" s="14">
         <f>SUMIFS($E$16:$E$24,$B$16:$B$24,"떡볶이")</f>
-        <v>394</v>
+        <v>431</v>
       </c>
       <c r="C30" s="9">
         <f>$D$9</f>
-        <v>271000</v>
+        <v>499000</v>
       </c>
       <c r="D30" s="9">
         <f>IF(B30=0,"",C30/B30)</f>
-        <v>687.81725888324877</v>
+        <v>1157.7726218097448</v>
       </c>
       <c r="E30" s="15">
-        <v>686838</v>
+        <v>1904431</v>
       </c>
       <c r="F30" s="16">
         <f>IFERROR( (E30 - (B30*D30)) / E30, "" )</f>
-        <v>0.60543825472673318</v>
+        <v>0.73797948048524731</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.35">
@@ -22586,22 +22853,22 @@
       </c>
       <c r="B31" s="14">
         <f>SUMIFS($E$16:$E$24,$B$16:$B$24,"꼬치오뎅")</f>
-        <v>652</v>
+        <v>738</v>
       </c>
       <c r="C31" s="9">
         <f>$D$10</f>
-        <v>194000</v>
+        <v>482400</v>
       </c>
       <c r="D31" s="9">
         <f>IF(B31=0,"",C31/B31)</f>
-        <v>297.54601226993867</v>
+        <v>653.65853658536582</v>
       </c>
       <c r="E31" s="15">
-        <v>690357</v>
+        <v>1769440</v>
       </c>
       <c r="F31" s="16">
         <f>IFERROR( (E31 - (B31*D31)) / E31, "" )</f>
-        <v>0.71898597392363661</v>
+        <v>0.72737137173342981</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.35">
@@ -22610,22 +22877,22 @@
       </c>
       <c r="B32" s="14">
         <f>SUMIFS($E$16:$E$24,$B$16:$B$24,"붕어빵")</f>
-        <v>3734</v>
+        <v>12470.5</v>
       </c>
       <c r="C32" s="9">
         <f>$D$11</f>
-        <v>904490</v>
+        <v>2658590</v>
       </c>
       <c r="D32" s="9">
         <f>IF(B32=0,"",C32/B32)</f>
-        <v>242.23085163363686</v>
+        <v>213.19032917685738</v>
       </c>
       <c r="E32" s="15">
-        <v>2457387</v>
+        <v>8351135</v>
       </c>
       <c r="F32" s="16">
         <f>IFERROR( (E32 - (B32*D32)) / E32, "" )</f>
-        <v>0.63193017624004688</v>
+        <v>0.68164926084897437</v>
       </c>
     </row>
     <row r="34" spans="1:6" ht="22.65" customHeight="1" x14ac:dyDescent="0.35">

</xml_diff>